<commit_message>
Work on brace and plate measurements
Changed the fft for brace and plates to be a shorter sample based on tap recognition. Also added harmonic analysis to pick the fundamentl. Also experimented with MPM (but it does not work well in this case).
Refactored TapToneAnalyzer to reduce file size and be better structured.
</commit_message>
<xml_diff>
--- a/Tests/Brace and Plate measurements.xlsx
+++ b/Tests/Brace and Plate measurements.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/dws/Library/CloudStorage/Dropbox/Programming/src/GuitarTap/Tests/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/dws/src/GuitarTap/Tests/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D564A21C-0FA7-A746-B686-85CE75705456}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{38B092F7-DFE4-D943-BA9C-625846B417E9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="820" yWindow="3320" windowWidth="28040" windowHeight="17180" xr2:uid="{67472550-BA94-354C-9432-C4165406051B}"/>
+    <workbookView xWindow="820" yWindow="2880" windowWidth="28040" windowHeight="17180" xr2:uid="{67472550-BA94-354C-9432-C4165406051B}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="11">
   <si>
     <t>Width</t>
   </si>
@@ -66,6 +66,9 @@
   </si>
   <si>
     <t>gm/cm^3</t>
+  </si>
+  <si>
+    <t>Bout Width</t>
   </si>
 </sst>
 </file>
@@ -95,7 +98,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -118,16 +121,33 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color rgb="FFA3A3A3"/>
+      </left>
+      <right style="medium">
+        <color rgb="FFA3A3A3"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -507,7 +527,7 @@
         <v>3</v>
       </c>
       <c r="B4" s="2">
-        <v>0.48499999999999999</v>
+        <v>4.8499999999999996</v>
       </c>
       <c r="C4" s="1" t="s">
         <v>1</v>
@@ -530,9 +550,35 @@
       <c r="A6" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="B6" s="1"/>
-      <c r="C6" s="1"/>
+      <c r="B6" s="1">
+        <v>0.34889999999999999</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>9</v>
+      </c>
       <c r="D6" s="1"/>
+    </row>
+    <row r="7" spans="1:4" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="B7" s="4">
+        <v>490</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="B8" s="4">
+        <v>368</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>1</v>
+      </c>
     </row>
     <row r="10" spans="1:4" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A10" t="s">

</xml_diff>

<commit_message>
feat(precision): FieldPrecision single source of truth + restrict-on-entry (Swift)
Add FieldPrecision — one decimal-count constant per field (table documented
in-code) + string()/rounded()/decimalsWithin() helpers. A limitedInput
binding rejects any keystroke beyond a field's P decimals on all 16 settings
fields, so an over-precise digit never appears (2-dp thickness takes 29.35,
not 29.356; a 0-decimal freq/dB field refuses the decimal point outright);
round-on-commit kept as a safety net. All seeds and the PDF Sample-Dimensions
rows format via the constant (Length/Width 1dp->2dp). Input, storage, and
display now agree per field. Build + 442 tests green.

@parity util/field-precision is a Swift-only orphan until the Python/web
mirrors land (PARITY-MAP regen to follow).

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Tests/Brace and Plate measurements.xlsx
+++ b/Tests/Brace and Plate measurements.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10222"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10719"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/dws/src/GuitarTap/Tests/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{38B092F7-DFE4-D943-BA9C-625846B417E9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8F6491CC-C846-3E48-89A6-AEC338E4943C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="820" yWindow="2880" windowWidth="28040" windowHeight="17180" xr2:uid="{67472550-BA94-354C-9432-C4165406051B}"/>
+    <workbookView xWindow="820" yWindow="1260" windowWidth="28040" windowHeight="17180" xr2:uid="{67472550-BA94-354C-9432-C4165406051B}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -98,7 +98,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="3">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -122,21 +122,38 @@
       <diagonal/>
     </border>
     <border>
-      <left style="medium">
-        <color rgb="FFA3A3A3"/>
+      <left style="thin">
+        <color indexed="64"/>
       </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
       <right style="medium">
         <color rgb="FFA3A3A3"/>
       </right>
-      <top/>
-      <bottom/>
+      <top style="medium">
+        <color rgb="FFA3A3A3"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FFA3A3A3"/>
+      </bottom>
       <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -144,10 +161,13 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -493,90 +513,90 @@
       </c>
     </row>
     <row r="2" spans="1:4" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="1" t="s">
+      <c r="A2" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="2">
+      <c r="B2" s="5">
         <v>220.5</v>
       </c>
-      <c r="C2" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="D2" s="1">
+      <c r="C2" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="D2" s="3">
         <f>B2*0.224</f>
         <v>49.392000000000003</v>
       </c>
     </row>
     <row r="3" spans="1:4" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="1" t="s">
+      <c r="A3" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="2">
+      <c r="B3" s="5">
         <v>557.5</v>
       </c>
-      <c r="C3" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="D3" s="1">
+      <c r="C3" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="D3" s="3">
         <f>B3*0.224</f>
         <v>124.88000000000001</v>
       </c>
     </row>
     <row r="4" spans="1:4" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="1" t="s">
+      <c r="A4" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="2">
+      <c r="B4" s="5">
         <v>4.8499999999999996</v>
       </c>
-      <c r="C4" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="D4" s="1"/>
+      <c r="C4" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="D4" s="3"/>
     </row>
     <row r="5" spans="1:4" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="1" t="s">
+      <c r="A5" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="B5" s="2">
+      <c r="B5" s="5">
         <v>208</v>
       </c>
-      <c r="C5" s="1" t="s">
+      <c r="C5" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="D5" s="1"/>
+      <c r="D5" s="3"/>
     </row>
     <row r="6" spans="1:4" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="1" t="s">
+      <c r="A6" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="B6" s="1">
+      <c r="B6" s="4">
         <v>0.34889999999999999</v>
       </c>
-      <c r="C6" s="1" t="s">
+      <c r="C6" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="D6" s="1"/>
-    </row>
-    <row r="7" spans="1:4" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="3" t="s">
+      <c r="D6" s="3"/>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A7" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="B7" s="4">
+      <c r="B7" s="5">
         <v>490</v>
       </c>
-      <c r="C7" s="1" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="3" t="s">
+      <c r="C7" s="4" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A8" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="B8" s="4">
+      <c r="B8" s="5">
         <v>368</v>
       </c>
-      <c r="C8" s="1" t="s">
+      <c r="C8" s="4" t="s">
         <v>1</v>
       </c>
     </row>

</xml_diff>